<commit_message>
Update BOM Calculator: Adjusted effective width now calculated as SB - effective width - 0.1
</commit_message>
<xml_diff>
--- a/data/Sources.xlsx
+++ b/data/Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfnonwovens-my.sharepoint.com/personal/mfischer_pfnonwovens_com/Documents/Desktop/mini-erp-node/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF32266F-029E-4EC8-8A76-FC6A52D9D36D}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="8_{66A118C3-EF46-4704-A6DB-C24509B266D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10397660-D5FC-4A7C-BD67-CAEFD81C45D4}"/>
   <bookViews>
-    <workbookView xWindow="34320" yWindow="21600" windowWidth="17415" windowHeight="20985" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
+    <workbookView xWindow="32910" yWindow="-8805" windowWidth="21600" windowHeight="12585" xr2:uid="{B924FA10-533B-4C07-A917-FCB6B882FB42}"/>
   </bookViews>
   <sheets>
     <sheet name="Lists" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="451">
   <si>
     <t>SB1</t>
   </si>
@@ -287,9 +287,6 @@
     <t>Buum</t>
   </si>
   <si>
-    <t xml:space="preserve">PLA </t>
-  </si>
-  <si>
     <t>070/30</t>
   </si>
   <si>
@@ -1383,6 +1380,27 @@
   </si>
   <si>
     <t>eC/S 5800</t>
+  </si>
+  <si>
+    <t>PET/coPET</t>
+  </si>
+  <si>
+    <t>PET/PP</t>
+  </si>
+  <si>
+    <t>G01 - Ovál</t>
+  </si>
+  <si>
+    <t>G09 - tulips</t>
+  </si>
+  <si>
+    <t>G11 - Spark</t>
+  </si>
+  <si>
+    <t>GXX - new</t>
+  </si>
+  <si>
+    <t>090/10</t>
   </si>
 </sst>
 </file>
@@ -1394,7 +1412,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1484,6 +1502,13 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="238"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1745,7 +1770,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1968,6 +1993,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1975,79 +2002,51 @@
   </cellStyles>
   <dxfs count="68">
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="none"/>
+      </font>
       <fill>
-        <patternFill>
-          <bgColor theme="4"/>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4"/>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3248,7 +3247,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="8"/>
-        <color theme="1"/>
+        <color auto="1"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -3259,6 +3258,7 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -3361,6 +3361,83 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="hair">
           <color theme="0" tint="-0.499984740745262"/>
@@ -3368,61 +3445,11 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <charset val="238"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border outline="0">
         <bottom style="hair">
           <color theme="0" tint="-0.499984740745262"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3554,187 +3581,193 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD2F10F3-78D8-42BB-8A3B-AA944E100804}" name="SB" displayName="SB" ref="A1:A31" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD2F10F3-78D8-42BB-8A3B-AA944E100804}" name="SB" displayName="SB" ref="A1:A31" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52" headerRowBorderDxfId="67" tableBorderDxfId="66" headerRowCellStyle="Normální 2">
   <autoFilter ref="A1:A31" xr:uid="{FD2F10F3-78D8-42BB-8A3B-AA944E100804}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{93E307B9-D269-4C9D-9138-FC89C896FC3D}" name="SB" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{93E307B9-D269-4C9D-9138-FC89C896FC3D}" name="SB" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}" name="Structure" displayName="Structure" ref="K1:K17" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}" name="Structure" displayName="Structure" ref="K1:K17" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" headerRowCellStyle="Normální 2">
   <autoFilter ref="K1:K17" xr:uid="{4905E39C-E898-4DCE-8992-EB9DD8BDD77C}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{56A23D9B-6A6F-4753-BE1E-C32EC840E0CC}" name="Structure" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{56A23D9B-6A6F-4753-BE1E-C32EC840E0CC}" name="Structure" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{413D5326-F5B7-47B4-B01A-6CB9BA8E80F3}" name="Main_RM" displayName="Main_RM" ref="L1:L20" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
-  <autoFilter ref="L1:L20" xr:uid="{413D5326-F5B7-47B4-B01A-6CB9BA8E80F3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{413D5326-F5B7-47B4-B01A-6CB9BA8E80F3}" name="Main_RM" displayName="Main_RM" ref="L1:L21" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+  <autoFilter ref="L1:L21" xr:uid="{413D5326-F5B7-47B4-B01A-6CB9BA8E80F3}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="L2:L21">
+    <sortCondition ref="L2:L22"/>
+  </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{DD8457DA-8491-478C-9906-5FD70BAC1D58}" name="Main RawMat" dataDxfId="32" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{DD8457DA-8491-478C-9906-5FD70BAC1D58}" name="Main RawMat" dataDxfId="23" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{1B04A6F5-7D60-4358-A04F-F7B790D5B889}" name="Bonding" displayName="Bonding" ref="M1:M13" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
-  <autoFilter ref="M1:M13" xr:uid="{1B04A6F5-7D60-4358-A04F-F7B790D5B889}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{1B04A6F5-7D60-4358-A04F-F7B790D5B889}" name="Bonding" displayName="Bonding" ref="M1:M17" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="M1:M17" xr:uid="{1B04A6F5-7D60-4358-A04F-F7B790D5B889}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{56ECAD42-4F9B-4A07-AFE4-7B55C7D60185}" name="Bonding" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{56ECAD42-4F9B-4A07-AFE4-7B55C7D60185}" name="Bonding" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FC924A71-2AB7-4534-BAF1-472867F8C212}" name="BICO_ratio" displayName="BICO_ratio" ref="N1:N11" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" headerRowCellStyle="Normální 2">
-  <autoFilter ref="N1:N11" xr:uid="{FC924A71-2AB7-4534-BAF1-472867F8C212}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FC924A71-2AB7-4534-BAF1-472867F8C212}" name="BICO_ratio" displayName="BICO_ratio" ref="N1:N12" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normální 2">
+  <autoFilter ref="N1:N12" xr:uid="{FC924A71-2AB7-4534-BAF1-472867F8C212}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N2:N12">
+    <sortCondition ref="N3:N12"/>
+  </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{328F5A89-E5FD-4981-8CDC-7C47CB509CD7}" name="BICO_ratio" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{328F5A89-E5FD-4981-8CDC-7C47CB509CD7}" name="BICO_ratio" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{C18F5E1C-F12C-48F7-8C94-ECB150008FB8}" name="Treatment" displayName="Treatment" ref="O1:O14" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{C18F5E1C-F12C-48F7-8C94-ECB150008FB8}" name="Treatment" displayName="Treatment" ref="O1:O14" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="O1:O14" xr:uid="{C18F5E1C-F12C-48F7-8C94-ECB150008FB8}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B95087BE-BB18-44FB-AB6B-CE34516E6A4E}" name="Treatment" dataDxfId="23" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{B95087BE-BB18-44FB-AB6B-CE34516E6A4E}" name="Treatment" dataDxfId="14" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{69417235-E692-4566-8941-350F0E308BFA}" name="Color" displayName="Color" ref="P1:P74" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{69417235-E692-4566-8941-350F0E308BFA}" name="Color" displayName="Color" ref="P1:P74" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="P1:P74" xr:uid="{69417235-E692-4566-8941-350F0E308BFA}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{D6D6BE17-33AB-4EE1-90CD-430533094C81}" name="Color" dataDxfId="20" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{D6D6BE17-33AB-4EE1-90CD-430533094C81}" name="Color" dataDxfId="11" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{8074344A-42F3-4096-BA1F-1011EBCE4F62}" name="Cores" displayName="Cores" ref="Q1:Q6" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{8074344A-42F3-4096-BA1F-1011EBCE4F62}" name="Cores" displayName="Cores" ref="Q1:Q6" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="Q1:Q6" xr:uid="{8074344A-42F3-4096-BA1F-1011EBCE4F62}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{D8816DF6-A4B5-48B7-95B8-92BAF88C9083}" name="Cores" dataDxfId="17" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{D8816DF6-A4B5-48B7-95B8-92BAF88C9083}" name="Cores" dataDxfId="8" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}" name="Line" displayName="Line" ref="R1:R14" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}" name="Line" displayName="Line" ref="R1:R14" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3" headerRowCellStyle="Normální 2" dataCellStyle="Normální 2">
   <autoFilter ref="R1:R14" xr:uid="{838775E4-F5E0-431D-9351-D17AE56F19D7}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{8390CAA7-046C-4F7E-8958-FFCCA51C7490}" name="Line" dataDxfId="14" dataCellStyle="Normální 2"/>
+    <tableColumn id="1" xr3:uid="{8390CAA7-046C-4F7E-8958-FFCCA51C7490}" name="Line" dataDxfId="5" dataCellStyle="Normální 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{CD1B2D88-330C-4AA5-92F9-DC81C83DDD5C}" name="Application" displayName="Application" ref="S1:S20" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{CD1B2D88-330C-4AA5-92F9-DC81C83DDD5C}" name="Application" displayName="Application" ref="S1:S20" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="S1:S20" xr:uid="{CD1B2D88-330C-4AA5-92F9-DC81C83DDD5C}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{07F71864-2ADD-444A-9722-A87171922B3B}" name="Application" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{07F71864-2ADD-444A-9722-A87171922B3B}" name="Application" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F86D69D5-51CA-46EE-92A0-1A2C34D527E8}" name="MB" displayName="MB" ref="B1:B7" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F86D69D5-51CA-46EE-92A0-1A2C34D527E8}" name="MB" displayName="MB" ref="B1:B7" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49" headerRowCellStyle="Normální 2">
   <autoFilter ref="B1:B7" xr:uid="{F86D69D5-51CA-46EE-92A0-1A2C34D527E8}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:B8">
     <sortCondition ref="B2:B8"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{11487E5B-596F-4AC8-82C2-4349BB217190}" name="MB" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{11487E5B-596F-4AC8-82C2-4349BB217190}" name="MB" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2B8E0AC4-5938-4202-A5F5-1FA75FC03C61}" name="Pigment" displayName="Pigment" ref="C1:C45" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2B8E0AC4-5938-4202-A5F5-1FA75FC03C61}" name="Pigment" displayName="Pigment" ref="C1:C45" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="C1:C45" xr:uid="{2B8E0AC4-5938-4202-A5F5-1FA75FC03C61}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{5FFC8618-1451-4571-84B4-2AAD5677FDAB}" name="Pigment" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{5FFC8618-1451-4571-84B4-2AAD5677FDAB}" name="Pigment" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CCCD4D2E-B90B-4A33-A594-ED7638EA8081}" name="Additive" displayName="Additive" ref="D1:D19" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CCCD4D2E-B90B-4A33-A594-ED7638EA8081}" name="Additive" displayName="Additive" ref="D1:D19" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="D1:D19" xr:uid="{CCCD4D2E-B90B-4A33-A594-ED7638EA8081}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{2DAF6286-B392-4B5E-91CB-F64910BE15E9}" name="Additive" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{2DAF6286-B392-4B5E-91CB-F64910BE15E9}" name="Additive" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium26" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4B7BC071-AFEA-40E1-A44E-F838AB3D3350}" name="Surfactant" displayName="Surfactant" ref="E1:F21" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4B7BC071-AFEA-40E1-A44E-F838AB3D3350}" name="Surfactant" displayName="Surfactant" ref="E1:F21" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="E1:F21" xr:uid="{4B7BC071-AFEA-40E1-A44E-F838AB3D3350}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{A58129B2-E318-4B2A-ADB4-7197D5F21149}" name="Surfactant" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{C14D571C-31A6-478E-8998-A5170562C0A0}" name="Surf_conc." dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{A58129B2-E318-4B2A-ADB4-7197D5F21149}" name="Surfactant" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{C14D571C-31A6-478E-8998-A5170562C0A0}" name="Surf_conc." dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{DFC0285C-169D-4176-8E8E-B72B97554CAF}" name="Customer" displayName="Customer" ref="G1:G87" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{DFC0285C-169D-4176-8E8E-B72B97554CAF}" name="Customer" displayName="Customer" ref="G1:G87" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="G1:G87" xr:uid="{DFC0285C-169D-4176-8E8E-B72B97554CAF}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{9356D4F7-572C-427C-AF1E-5EB78F6FE98E}" name="Customer" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{9356D4F7-572C-427C-AF1E-5EB78F6FE98E}" name="Customer" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{900597CB-2276-43CA-8635-9ED863BCF790}" name="Segment" displayName="Segment" ref="H1:H7" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{900597CB-2276-43CA-8635-9ED863BCF790}" name="Segment" displayName="Segment" ref="H1:H7" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33" headerRowCellStyle="Normální 2">
   <autoFilter ref="H1:H7" xr:uid="{900597CB-2276-43CA-8635-9ED863BCF790}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{938C3C67-4ACA-4662-9C57-E897A4B22B13}" name="Segment" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{938C3C67-4ACA-4662-9C57-E897A4B22B13}" name="Segment" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}" name="S_SMS" displayName="S_SMS" ref="I1:I6" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}" name="S_SMS" displayName="S_SMS" ref="I1:I6" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30" headerRowCellStyle="Normální 2">
   <autoFilter ref="I1:I6" xr:uid="{6464D72C-C69A-4112-8424-97766E88D7C7}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{139A78FA-5925-4655-AE99-194FDAFDFE73}" name="S/SMS" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{139A78FA-5925-4655-AE99-194FDAFDFE73}" name="S/SMS" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6F590121-595E-4041-9C49-F227887713EB}" name="Mono_Bico" displayName="Mono_Bico" ref="J1:J4" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39" headerRowCellStyle="Normální 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6F590121-595E-4041-9C49-F227887713EB}" name="Mono_Bico" displayName="Mono_Bico" ref="J1:J4" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" headerRowCellStyle="Normální 2">
   <autoFilter ref="J1:J4" xr:uid="{6F590121-595E-4041-9C49-F227887713EB}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J2:J4">
     <sortCondition descending="1" ref="J2:J4"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{49BE5F34-76EF-4FC6-AD85-4A01D164CFDE}" name="Mono/Bico" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{49BE5F34-76EF-4FC6-AD85-4A01D164CFDE}" name="Mono/Bico" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium24" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4057,7 +4090,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB1CF6A9-7DDA-404E-90FB-FA3DB2C74227}">
-  <dimension ref="A1:AD3514"/>
+  <dimension ref="A1:AD3506"/>
   <sheetFormatPr defaultColWidth="7.109375" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="25.77734375" style="5" customWidth="1"/>
@@ -4081,46 +4114,46 @@
   <sheetData>
     <row r="1" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="57" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>271</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>272</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="O1" s="4" t="s">
         <v>8</v>
@@ -4132,7 +4165,7 @@
         <v>9</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>10</v>
@@ -4140,19 +4173,19 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F2" s="8">
         <v>1</v>
@@ -4178,8 +4211,8 @@
       <c r="M2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="7" t="s">
-        <v>277</v>
+      <c r="N2" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="O2" s="7" t="s">
         <v>19</v>
@@ -4199,19 +4232,19 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F3" s="8">
         <v>1</v>
@@ -4238,7 +4271,7 @@
         <v>23</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="O3" s="7" t="s">
         <v>31</v>
@@ -4258,19 +4291,19 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F4" s="8">
         <v>0.99</v>
@@ -4288,7 +4321,7 @@
         <v>14</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>40</v>
@@ -4297,7 +4330,7 @@
         <v>41</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="O4" s="7" t="s">
         <v>43</v>
@@ -4317,19 +4350,19 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F5" s="8">
         <v>1</v>
@@ -4350,10 +4383,10 @@
         <v>52</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="O5" s="7" t="s">
         <v>54</v>
@@ -4373,19 +4406,19 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F6" s="8">
         <v>0.5</v>
@@ -4400,16 +4433,16 @@
         <v>61</v>
       </c>
       <c r="K6" s="68" t="s">
-        <v>433</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>62</v>
+        <v>432</v>
+      </c>
+      <c r="L6" s="69" t="s">
+        <v>444</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>63</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>65</v>
@@ -4429,19 +4462,19 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F7" s="8">
         <v>1</v>
@@ -4450,19 +4483,19 @@
         <v>70</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="K7" s="68" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="M7" s="5" t="s">
         <v>72</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="O7" s="7" t="s">
         <v>74</v>
@@ -4479,16 +4512,16 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F8" s="8">
         <v>1</v>
@@ -4497,69 +4530,69 @@
         <v>78</v>
       </c>
       <c r="K8" s="68" t="s">
-        <v>435</v>
-      </c>
-      <c r="L8" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="L8" s="69" t="s">
+        <v>445</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="N8" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M8" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="N8" s="5" t="s">
-        <v>73</v>
-      </c>
       <c r="O8" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="P8" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="R8" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="R8" s="7" t="s">
+      <c r="S8" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="S8" s="5" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F9" s="8">
         <v>0.45</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K9" s="68" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="L9" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="M9" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="N9" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="N9" s="5" t="s">
-        <v>80</v>
-      </c>
       <c r="O9" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="P9" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="P9" s="7" t="s">
+      <c r="R9" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="R9" s="7" t="s">
-        <v>91</v>
       </c>
       <c r="S9" s="5" t="s">
         <v>15</v>
@@ -4567,1109 +4600,1135 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F10" s="8">
         <v>0.94</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K10" s="68" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="N10" s="5" t="s">
-        <v>88</v>
+        <v>392</v>
+      </c>
+      <c r="N10" s="68" t="s">
+        <v>450</v>
       </c>
       <c r="O10" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="P10" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="P10" s="7" t="s">
+      <c r="R10" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="R10" s="7" t="s">
+      <c r="S10" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="S10" s="5" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F11" s="8">
         <v>0.43</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K11" s="68" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="L11" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="O11" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="M11" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="O11" s="7" t="s">
+      <c r="P11" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="7" t="s">
+      <c r="R11" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="R11" s="7" t="s">
+      <c r="S11" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="S11" s="5" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F12" s="8">
         <v>0.5</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K12" s="68" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="L12" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="M12" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="M12" s="5" t="s">
+      <c r="N12" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="O12" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="O12" s="7" t="s">
+      <c r="P12" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="P12" s="7" t="s">
+      <c r="R12" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="R12" s="7" t="s">
+      <c r="S12" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="S12" s="5" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F13" s="8">
         <v>0.5</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K13" s="68" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L13" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M13" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="M13" s="5" t="s">
+      <c r="O13" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="O13" s="7" t="s">
+      <c r="P13" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="7" t="s">
+      <c r="R13" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="R13" s="7" t="s">
+      <c r="S13" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="S13" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F14" s="8">
         <v>0.76</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K14" s="68" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="L14" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="M14" s="68" t="s">
+        <v>446</v>
+      </c>
+      <c r="O14" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="O14" s="7" t="s">
+      <c r="P14" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="P14" s="7" t="s">
+      <c r="R14" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="R14" s="7" t="s">
+      <c r="S14" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="S14" s="5" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F15" s="8">
         <v>0.96</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K15" s="68" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="L15" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M15" s="68" t="s">
+        <v>447</v>
+      </c>
+      <c r="P15" s="7" t="s">
         <v>126</v>
-      </c>
-      <c r="P15" s="7" t="s">
-        <v>127</v>
       </c>
       <c r="R15" s="7"/>
       <c r="S15" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F16" s="8">
         <v>0.19</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K16" s="68" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="L16" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="M16" s="68" t="s">
+        <v>448</v>
+      </c>
+      <c r="P16" s="7" t="s">
         <v>130</v>
-      </c>
-      <c r="P16" s="7" t="s">
-        <v>131</v>
       </c>
       <c r="R16" s="7"/>
       <c r="S16" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F17" s="8">
         <v>0.2</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K17" s="68" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="L17" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="M17" s="68" t="s">
+        <v>449</v>
+      </c>
+      <c r="P17" s="7" t="s">
         <v>134</v>
-      </c>
-      <c r="P17" s="7" t="s">
-        <v>135</v>
       </c>
       <c r="R17" s="7"/>
       <c r="S17" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F18" s="8">
         <v>0.6</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L18" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="M18" s="70"/>
+      <c r="P18" s="7" t="s">
         <v>138</v>
-      </c>
-      <c r="P18" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="R18" s="7"/>
       <c r="S18" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F19" s="8">
         <v>1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L19" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="M19" s="70"/>
+      <c r="P19" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="P19" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F20" s="8">
         <v>0.03</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="L20" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="M20" s="70"/>
+      <c r="P20" s="7" t="s">
         <v>146</v>
-      </c>
-      <c r="P20" s="7" t="s">
-        <v>147</v>
       </c>
       <c r="R20" s="7"/>
       <c r="S20" s="5" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F21" s="8">
         <v>0.7</v>
       </c>
       <c r="G21" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="M21" s="70"/>
+      <c r="P21" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="L21" s="7"/>
-      <c r="P21" s="7" t="s">
-        <v>149</v>
-      </c>
       <c r="R21" s="7"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="L22" s="70"/>
+      <c r="M22" s="70"/>
+      <c r="P22" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="L22" s="7"/>
-      <c r="P22" s="7" t="s">
-        <v>151</v>
-      </c>
       <c r="R22" s="7"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="L23" s="70"/>
+      <c r="M23" s="70"/>
+      <c r="P23" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="L23" s="7"/>
-      <c r="P23" s="7" t="s">
-        <v>153</v>
-      </c>
       <c r="R23" s="7"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="L24" s="70"/>
+      <c r="M24" s="70"/>
+      <c r="P24" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="L24" s="7"/>
-      <c r="P24" s="7" t="s">
-        <v>155</v>
-      </c>
       <c r="R24" s="7"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="L25" s="70"/>
+      <c r="M25" s="70"/>
+      <c r="P25" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="L25" s="7"/>
-      <c r="P25" s="7" t="s">
-        <v>157</v>
-      </c>
       <c r="R25" s="7"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="L26" s="70"/>
+      <c r="M26" s="70"/>
+      <c r="P26" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="L26" s="7"/>
-      <c r="P26" s="7" t="s">
-        <v>159</v>
-      </c>
       <c r="R26" s="7"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="L27" s="70"/>
+      <c r="P27" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="L27" s="7"/>
-      <c r="P27" s="7" t="s">
-        <v>161</v>
-      </c>
       <c r="R27" s="7"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="L28" s="70"/>
+      <c r="P28" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="L28" s="7"/>
-      <c r="P28" s="7" t="s">
-        <v>163</v>
-      </c>
       <c r="R28" s="7"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="L29" s="70"/>
+      <c r="P29" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="L29" s="7"/>
-      <c r="P29" s="7" t="s">
-        <v>165</v>
-      </c>
       <c r="R29" s="7"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="L30" s="70"/>
+      <c r="P30" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="L30" s="7"/>
-      <c r="P30" s="7" t="s">
-        <v>167</v>
-      </c>
       <c r="R30" s="7"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="L31" s="70"/>
+      <c r="P31" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="L31" s="7"/>
-      <c r="P31" s="7" t="s">
-        <v>169</v>
-      </c>
       <c r="R31" s="7"/>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C32" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="L32" s="70"/>
+      <c r="P32" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="L32" s="7"/>
-      <c r="P32" s="7" t="s">
-        <v>171</v>
-      </c>
       <c r="R32" s="7"/>
     </row>
-    <row r="33" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="33" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C33" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="L33" s="70"/>
+      <c r="P33" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="L33" s="7"/>
-      <c r="P33" s="7" t="s">
-        <v>173</v>
-      </c>
       <c r="R33" s="7"/>
     </row>
-    <row r="34" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C34" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="L34" s="70"/>
+      <c r="P34" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="L34" s="7"/>
-      <c r="P34" s="7" t="s">
-        <v>175</v>
-      </c>
       <c r="R34" s="7"/>
     </row>
-    <row r="35" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C35" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="L35" s="70"/>
+      <c r="P35" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="L35" s="7"/>
-      <c r="P35" s="7" t="s">
-        <v>177</v>
-      </c>
       <c r="R35" s="7"/>
     </row>
-    <row r="36" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="36" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C36" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="L36" s="70"/>
+      <c r="P36" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="L36" s="7"/>
-      <c r="P36" s="7" t="s">
-        <v>179</v>
-      </c>
       <c r="R36" s="7"/>
     </row>
-    <row r="37" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C37" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="L37" s="70"/>
+      <c r="P37" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="L37" s="7"/>
-      <c r="P37" s="7" t="s">
-        <v>181</v>
-      </c>
       <c r="R37" s="7"/>
     </row>
-    <row r="38" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C38" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="L38" s="70"/>
+      <c r="P38" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="L38" s="7"/>
-      <c r="P38" s="7" t="s">
-        <v>183</v>
-      </c>
       <c r="R38" s="7"/>
     </row>
-    <row r="39" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="39" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C39" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="L39" s="70"/>
+      <c r="P39" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="L39" s="7"/>
-      <c r="P39" s="7" t="s">
-        <v>185</v>
-      </c>
       <c r="R39" s="7"/>
     </row>
-    <row r="40" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C40" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="L40" s="70"/>
+      <c r="P40" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="L40" s="7"/>
-      <c r="P40" s="7" t="s">
-        <v>187</v>
-      </c>
       <c r="R40" s="7"/>
     </row>
-    <row r="41" spans="3:18" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:18" ht="10.8" x14ac:dyDescent="0.25">
       <c r="C41" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="L41" s="70"/>
+      <c r="P41" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="L41" s="7"/>
-      <c r="P41" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="R41" s="7"/>
     </row>
     <row r="42" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C42" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L42" s="7"/>
       <c r="P42" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="R42" s="7"/>
     </row>
     <row r="43" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C43" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L43" s="7"/>
       <c r="P43" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R43" s="7"/>
     </row>
     <row r="44" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C44" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="L44" s="7"/>
       <c r="P44" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="R44" s="7"/>
     </row>
     <row r="45" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C45" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L45" s="7"/>
       <c r="P45" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="R45" s="7"/>
     </row>
     <row r="46" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F46" s="6"/>
       <c r="G46" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="L46" s="7"/>
       <c r="P46" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="R46" s="7"/>
     </row>
     <row r="47" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F47" s="6"/>
       <c r="G47" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L47" s="7"/>
       <c r="P47" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="R47" s="7"/>
     </row>
     <row r="48" spans="3:18" x14ac:dyDescent="0.2">
       <c r="F48" s="6"/>
       <c r="G48" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L48" s="7"/>
       <c r="P48" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="R48" s="7"/>
     </row>
     <row r="49" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F49" s="6"/>
       <c r="G49" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L49" s="7"/>
       <c r="P49" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="R49" s="7"/>
     </row>
     <row r="50" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F50" s="6"/>
       <c r="G50" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="L50" s="7"/>
       <c r="P50" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="R50" s="7"/>
     </row>
     <row r="51" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F51" s="6"/>
       <c r="G51" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="L51" s="7"/>
       <c r="P51" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="R51" s="7"/>
     </row>
     <row r="52" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F52" s="6"/>
       <c r="G52" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L52" s="7"/>
       <c r="P52" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="R52" s="7"/>
     </row>
     <row r="53" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F53" s="6"/>
       <c r="G53" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L53" s="7"/>
       <c r="P53" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="R53" s="7"/>
     </row>
     <row r="54" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F54" s="6"/>
       <c r="G54" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="L54" s="7"/>
       <c r="P54" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="R54" s="7"/>
     </row>
     <row r="55" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F55" s="6"/>
       <c r="G55" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="L55" s="7"/>
       <c r="P55" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="R55" s="7"/>
     </row>
     <row r="56" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F56" s="6"/>
       <c r="G56" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L56" s="7"/>
       <c r="P56" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="R56" s="7"/>
     </row>
     <row r="57" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F57" s="6"/>
       <c r="G57" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="L57" s="7"/>
       <c r="P57" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="R57" s="7"/>
     </row>
     <row r="58" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F58" s="6"/>
       <c r="G58" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="L58" s="7"/>
       <c r="P58" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="R58" s="7"/>
     </row>
     <row r="59" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F59" s="6"/>
       <c r="G59" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="L59" s="7"/>
       <c r="P59" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R59" s="7"/>
     </row>
     <row r="60" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F60" s="6"/>
       <c r="G60" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L60" s="7"/>
       <c r="P60" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="R60" s="7"/>
     </row>
     <row r="61" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F61" s="6"/>
       <c r="G61" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L61" s="7"/>
       <c r="P61" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="R61" s="7"/>
     </row>
     <row r="62" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F62" s="6"/>
       <c r="G62" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L62" s="7"/>
       <c r="P62" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="R62" s="7"/>
     </row>
     <row r="63" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F63" s="6"/>
       <c r="G63" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="L63" s="7"/>
       <c r="P63" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R63" s="7"/>
     </row>
     <row r="64" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F64" s="6"/>
       <c r="G64" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L64" s="7"/>
       <c r="P64" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R64" s="7"/>
     </row>
     <row r="65" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F65" s="6"/>
       <c r="G65" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="L65" s="7"/>
       <c r="P65" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="R65" s="7"/>
     </row>
     <row r="66" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F66" s="6"/>
       <c r="G66" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L66" s="7"/>
       <c r="P66" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="R66" s="7"/>
     </row>
     <row r="67" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F67" s="6"/>
       <c r="G67" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L67" s="7"/>
       <c r="P67" s="7" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="R67" s="7"/>
     </row>
     <row r="68" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F68" s="6"/>
       <c r="G68" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L68" s="7"/>
       <c r="P68" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="R68" s="7"/>
     </row>
     <row r="69" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F69" s="6"/>
       <c r="G69" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="L69" s="7"/>
       <c r="P69" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="R69" s="7"/>
     </row>
     <row r="70" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F70" s="6"/>
       <c r="G70" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="L70" s="7"/>
       <c r="P70" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="R70" s="7"/>
     </row>
     <row r="71" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F71" s="6"/>
       <c r="G71" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="L71" s="7"/>
       <c r="P71" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="R71" s="7"/>
     </row>
     <row r="72" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F72" s="6"/>
       <c r="G72" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="L72" s="7"/>
       <c r="P72" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="R72" s="7"/>
     </row>
     <row r="73" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F73" s="6"/>
       <c r="G73" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="L73" s="7"/>
       <c r="P73" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="R73" s="7"/>
     </row>
     <row r="74" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F74" s="6"/>
       <c r="G74" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="L74" s="7"/>
       <c r="P74" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="R74" s="7"/>
     </row>
     <row r="75" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F75" s="6"/>
       <c r="G75" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="L75" s="7"/>
       <c r="R75" s="7"/>
@@ -5677,7 +5736,7 @@
     <row r="76" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F76" s="6"/>
       <c r="G76" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="L76" s="7"/>
       <c r="R76" s="7"/>
@@ -5685,7 +5744,7 @@
     <row r="77" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F77" s="6"/>
       <c r="G77" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="L77" s="7"/>
       <c r="R77" s="7"/>
@@ -5693,7 +5752,7 @@
     <row r="78" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F78" s="6"/>
       <c r="G78" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="L78" s="7"/>
       <c r="R78" s="7"/>
@@ -5701,7 +5760,7 @@
     <row r="79" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F79" s="6"/>
       <c r="G79" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L79" s="7"/>
       <c r="R79" s="7"/>
@@ -5709,7 +5768,7 @@
     <row r="80" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F80" s="6"/>
       <c r="G80" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L80" s="7"/>
       <c r="R80" s="7"/>
@@ -5717,7 +5776,7 @@
     <row r="81" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F81" s="6"/>
       <c r="G81" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L81" s="7"/>
       <c r="R81" s="7"/>
@@ -5725,7 +5784,7 @@
     <row r="82" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F82" s="6"/>
       <c r="G82" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L82" s="7"/>
       <c r="R82" s="7"/>
@@ -5733,7 +5792,7 @@
     <row r="83" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F83" s="6"/>
       <c r="G83" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="L83" s="7"/>
       <c r="R83" s="7"/>
@@ -5741,7 +5800,7 @@
     <row r="84" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F84" s="6"/>
       <c r="G84" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="L84" s="7"/>
       <c r="R84" s="7"/>
@@ -5749,7 +5808,7 @@
     <row r="85" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F85" s="6"/>
       <c r="G85" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="L85" s="7"/>
       <c r="R85" s="7"/>
@@ -5757,7 +5816,7 @@
     <row r="86" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F86" s="6"/>
       <c r="G86" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="L86" s="7"/>
       <c r="R86" s="7"/>
@@ -5765,7 +5824,7 @@
     <row r="87" spans="6:18" x14ac:dyDescent="0.2">
       <c r="F87" s="6"/>
       <c r="G87" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L87" s="7"/>
       <c r="R87" s="7"/>
@@ -5785,34 +5844,33 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="3514" spans="30:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G2:G87">
     <sortCondition ref="G2:G87"/>
   </sortState>
   <conditionalFormatting sqref="A15:A17">
-    <cfRule type="duplicateValues" dxfId="10" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18">
-    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B87">
-    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C87">
-    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D24 D26:D87 A22">
-    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18">
-    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13">
-    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G87">
-    <cfRule type="duplicateValues" dxfId="3" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="9"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="18">
@@ -5857,7 +5915,7 @@
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="9"/>
       <c r="B1" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
@@ -5892,7 +5950,7 @@
         <v>1000</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
@@ -5922,11 +5980,11 @@
       <c r="A3" s="10"/>
       <c r="B3" s="10"/>
       <c r="C3" s="58" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D3" s="59"/>
       <c r="E3" s="58" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F3" s="59"/>
       <c r="G3" s="14" t="s">
@@ -5942,11 +6000,11 @@
         <v>13</v>
       </c>
       <c r="K3" s="60" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="L3" s="61"/>
       <c r="M3" s="58" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N3" s="59"/>
       <c r="O3" s="9"/>
@@ -5965,35 +6023,35 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="62" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D4" s="63"/>
       <c r="E4" s="62" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F4" s="63"/>
       <c r="G4" s="17" t="s">
+        <v>398</v>
+      </c>
+      <c r="H4" s="15" t="s">
         <v>399</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="I4" s="17" t="s">
         <v>400</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="J4" s="15" t="s">
         <v>401</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="K4" s="62" t="s">
         <v>402</v>
-      </c>
-      <c r="K4" s="62" t="s">
-        <v>403</v>
       </c>
       <c r="L4" s="63"/>
       <c r="M4" s="62" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="N4" s="63"/>
       <c r="O4" s="9"/>
@@ -6012,7 +6070,7 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B5" s="18"/>
       <c r="C5" s="64">
@@ -6050,7 +6108,7 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B6" s="25"/>
       <c r="C6" s="66">
@@ -6108,44 +6166,44 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B7" s="29"/>
       <c r="C7" s="30" t="s">
+        <v>407</v>
+      </c>
+      <c r="D7" s="30" t="s">
         <v>408</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="E7" s="30" t="s">
+        <v>407</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>408</v>
+      </c>
+      <c r="G7" s="30" t="s">
         <v>409</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="H7" s="30" t="s">
+        <v>409</v>
+      </c>
+      <c r="I7" s="30" t="s">
+        <v>409</v>
+      </c>
+      <c r="J7" s="30" t="s">
+        <v>409</v>
+      </c>
+      <c r="K7" s="30" t="s">
+        <v>407</v>
+      </c>
+      <c r="L7" s="30" t="s">
         <v>408</v>
       </c>
-      <c r="F7" s="30" t="s">
-        <v>409</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>410</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>410</v>
-      </c>
-      <c r="I7" s="30" t="s">
-        <v>410</v>
-      </c>
-      <c r="J7" s="30" t="s">
-        <v>410</v>
-      </c>
-      <c r="K7" s="30" t="s">
+      <c r="M7" s="30" t="s">
+        <v>407</v>
+      </c>
+      <c r="N7" s="30" t="s">
         <v>408</v>
-      </c>
-      <c r="L7" s="30" t="s">
-        <v>409</v>
-      </c>
-      <c r="M7" s="30" t="s">
-        <v>408</v>
-      </c>
-      <c r="N7" s="30" t="s">
-        <v>409</v>
       </c>
       <c r="O7" s="9"/>
       <c r="P7" s="9"/>
@@ -6163,7 +6221,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B8" s="29"/>
       <c r="C8" s="32">
@@ -6261,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C10" s="32">
         <v>1</v>
@@ -6343,7 +6401,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B12" s="32"/>
       <c r="C12" s="37"/>
@@ -6418,7 +6476,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="29" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B14" s="32"/>
       <c r="C14" s="37"/>
@@ -6491,10 +6549,10 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B16" s="32" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C16" s="37">
         <v>7.0000000000000001E-3</v>
@@ -6526,7 +6584,7 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B17" s="32"/>
       <c r="C17" s="37"/>
@@ -6557,7 +6615,7 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="37"/>
@@ -6588,7 +6646,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B19" s="32"/>
       <c r="C19" s="37"/>
@@ -6619,7 +6677,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" s="29" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B20" s="32"/>
       <c r="C20" s="37"/>
@@ -6681,13 +6739,13 @@
       <c r="A22" s="41"/>
       <c r="B22" s="42"/>
       <c r="C22" s="43" t="s">
+        <v>418</v>
+      </c>
+      <c r="D22" s="43" t="s">
         <v>419</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="E22" s="44" t="s">
         <v>420</v>
-      </c>
-      <c r="E22" s="44" t="s">
-        <v>421</v>
       </c>
       <c r="F22" s="45"/>
       <c r="G22" s="45"/>
@@ -6714,10 +6772,10 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" s="29" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B23" s="32" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C23" s="35">
         <f>_xlfn.XLOOKUP(B23,Surfactant[Surfactant],Surfactant[Surf_conc.])</f>
@@ -6755,7 +6813,7 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" s="29" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B24" s="32"/>
       <c r="C24" s="35" t="e">
@@ -6792,7 +6850,7 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" s="29" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="35" t="e">
@@ -6861,76 +6919,76 @@
         <v>0</v>
       </c>
       <c r="B27" s="48" t="s">
+        <v>411</v>
+      </c>
+      <c r="C27" s="48" t="s">
         <v>412</v>
-      </c>
-      <c r="C27" s="48" t="s">
-        <v>413</v>
       </c>
       <c r="D27" s="48" t="s">
         <v>1</v>
       </c>
       <c r="E27" s="48" t="s">
+        <v>413</v>
+      </c>
+      <c r="F27" s="48" t="s">
         <v>414</v>
       </c>
-      <c r="F27" s="48" t="s">
+      <c r="G27" s="48" t="s">
         <v>415</v>
       </c>
-      <c r="G27" s="48" t="s">
+      <c r="H27" s="48" t="s">
         <v>416</v>
       </c>
-      <c r="H27" s="48" t="s">
+      <c r="I27" s="48" t="s">
         <v>417</v>
       </c>
-      <c r="I27" s="48" t="s">
-        <v>418</v>
-      </c>
       <c r="J27" s="48" t="s">
+        <v>421</v>
+      </c>
+      <c r="K27" s="48" t="s">
         <v>422</v>
       </c>
-      <c r="K27" s="48" t="s">
+      <c r="L27" s="48" t="s">
         <v>423</v>
-      </c>
-      <c r="L27" s="48" t="s">
-        <v>424</v>
       </c>
       <c r="M27" s="48" t="s">
         <v>0</v>
       </c>
       <c r="N27" s="48" t="s">
+        <v>411</v>
+      </c>
+      <c r="O27" s="48" t="s">
         <v>412</v>
-      </c>
-      <c r="O27" s="48" t="s">
-        <v>413</v>
       </c>
       <c r="P27" s="48" t="s">
         <v>1</v>
       </c>
       <c r="Q27" s="48" t="s">
+        <v>413</v>
+      </c>
+      <c r="R27" s="48" t="s">
         <v>414</v>
       </c>
-      <c r="R27" s="48" t="s">
+      <c r="S27" s="48" t="s">
         <v>415</v>
       </c>
-      <c r="S27" s="48" t="s">
+      <c r="T27" s="48" t="s">
         <v>416</v>
       </c>
-      <c r="T27" s="48" t="s">
+      <c r="U27" s="48" t="s">
         <v>417</v>
       </c>
-      <c r="U27" s="48" t="s">
-        <v>418</v>
-      </c>
       <c r="V27" s="48" t="s">
+        <v>421</v>
+      </c>
+      <c r="W27" s="48" t="s">
         <v>422</v>
       </c>
-      <c r="W27" s="48" t="s">
+      <c r="X27" s="48" t="s">
         <v>423</v>
       </c>
-      <c r="X27" s="48" t="s">
-        <v>424</v>
-      </c>
       <c r="Y27" s="48" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="Z27" s="22"/>
       <c r="AA27" s="22"/>
@@ -7106,15 +7164,15 @@
     <mergeCell ref="M4:N4"/>
   </mergeCells>
   <conditionalFormatting sqref="A29">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="notEqual">
+    <cfRule type="cellIs" dxfId="57" priority="1" operator="notEqual">
       <formula>1000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="2" operator="equal">
       <formula>1000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="4"/>
   </conditionalFormatting>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10:B14" xr:uid="{0004E0DC-B181-412E-9546-AF22382DF408}">

</xml_diff>